<commit_message>
Actualización del archivo Python
</commit_message>
<xml_diff>
--- a/datos_Grup C.xlsx
+++ b/datos_Grup C.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U138"/>
+  <dimension ref="A1:S138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,16 +525,6 @@
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>Increment_x</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Increment_y</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
           <t>Increment</t>
         </is>
       </c>
@@ -604,7 +594,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>2563.55</v>
+        <v>2513.28</v>
       </c>
       <c r="Q2" s="2" t="n">
         <v>31778</v>
@@ -615,14 +605,6 @@
       <c r="S2" t="n">
         <v>0.02</v>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U2" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -685,7 +667,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>2117.21</v>
+        <v>2075.7</v>
       </c>
       <c r="Q3" s="2" t="n">
         <v>31943</v>
@@ -696,14 +678,6 @@
       <c r="S3" t="n">
         <v>0.02</v>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U3" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -770,7 +744,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>2541.7</v>
+        <v>2491.86</v>
       </c>
       <c r="Q4" s="2" t="n">
         <v>31181</v>
@@ -781,14 +755,6 @@
       <c r="S4" t="n">
         <v>0.02</v>
       </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U4" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -855,7 +821,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>2050.63</v>
+        <v>2010.42</v>
       </c>
       <c r="Q5" s="2" t="n">
         <v>18921</v>
@@ -866,14 +832,6 @@
       <c r="S5" t="n">
         <v>0.02</v>
       </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U5" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -940,7 +898,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>2688.39</v>
+        <v>2635.68</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>31522</v>
@@ -951,14 +909,6 @@
       <c r="S6" t="n">
         <v>0.02</v>
       </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U6" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1025,7 +975,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>2581.23</v>
+        <v>2530.62</v>
       </c>
       <c r="Q7" s="2" t="n">
         <v>21436</v>
@@ -1036,14 +986,6 @@
       <c r="S7" t="n">
         <v>0.02</v>
       </c>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U7" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1110,7 +1052,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>1753.07</v>
+        <v>1718.7</v>
       </c>
       <c r="Q8" s="2" t="n">
         <v>34616</v>
@@ -1121,14 +1063,6 @@
       <c r="S8" t="n">
         <v>0.02</v>
       </c>
-      <c r="T8" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U8" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1195,7 +1129,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>2701.92</v>
+        <v>2648.94</v>
       </c>
       <c r="Q9" s="2" t="n">
         <v>18873</v>
@@ -1206,14 +1140,6 @@
       <c r="S9" t="n">
         <v>0.02</v>
       </c>
-      <c r="T9" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U9" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1280,7 +1206,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>2763.3</v>
+        <v>2709.12</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>19887</v>
@@ -1291,14 +1217,6 @@
       <c r="S10" t="n">
         <v>0.02</v>
       </c>
-      <c r="T10" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U10" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1365,7 +1283,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>2748.74</v>
+        <v>2694.84</v>
       </c>
       <c r="Q11" s="2" t="n">
         <v>18817</v>
@@ -1376,14 +1294,6 @@
       <c r="S11" t="n">
         <v>0.02</v>
       </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U11" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1450,7 +1360,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>2112.01</v>
+        <v>2070.6</v>
       </c>
       <c r="Q12" s="2" t="n">
         <v>19760</v>
@@ -1461,14 +1371,6 @@
       <c r="S12" t="n">
         <v>0.02</v>
       </c>
-      <c r="T12" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U12" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1535,7 +1437,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>2793.47</v>
+        <v>2738.7</v>
       </c>
       <c r="Q13" s="2" t="n">
         <v>31489</v>
@@ -1546,14 +1448,6 @@
       <c r="S13" t="n">
         <v>0.02</v>
       </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U13" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1620,7 +1514,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>2493.84</v>
+        <v>2444.94</v>
       </c>
       <c r="Q14" s="2" t="n">
         <v>27292</v>
@@ -1631,14 +1525,6 @@
       <c r="S14" t="n">
         <v>0.02</v>
       </c>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U14" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1705,7 +1591,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>2745.62</v>
+        <v>2691.78</v>
       </c>
       <c r="Q15" s="2" t="n">
         <v>31149</v>
@@ -1716,14 +1602,6 @@
       <c r="S15" t="n">
         <v>0.02</v>
       </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U15" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1790,7 +1668,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>2551.06</v>
+        <v>2501.04</v>
       </c>
       <c r="Q16" s="2" t="n">
         <v>28322</v>
@@ -1801,14 +1679,6 @@
       <c r="S16" t="n">
         <v>0.02</v>
       </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U16" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1875,7 +1745,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>2649.9</v>
+        <v>2597.94</v>
       </c>
       <c r="Q17" s="2" t="n">
         <v>19142</v>
@@ -1886,14 +1756,6 @@
       <c r="S17" t="n">
         <v>0.02</v>
       </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U17" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1960,7 +1822,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>2297.2</v>
+        <v>2252.16</v>
       </c>
       <c r="Q18" s="2" t="n">
         <v>31434</v>
@@ -1971,14 +1833,6 @@
       <c r="S18" t="n">
         <v>0.02</v>
       </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U18" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2045,7 +1899,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>2835.09</v>
+        <v>2779.5</v>
       </c>
       <c r="Q19" s="2" t="n">
         <v>36417</v>
@@ -2056,14 +1910,6 @@
       <c r="S19" t="n">
         <v>0.02</v>
       </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U19" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2130,7 +1976,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>2017.34</v>
+        <v>1977.78</v>
       </c>
       <c r="Q20" s="2" t="n">
         <v>29756</v>
@@ -2141,14 +1987,6 @@
       <c r="S20" t="n">
         <v>0.02</v>
       </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U20" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2215,7 +2053,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>2901.68</v>
+        <v>2844.78</v>
       </c>
       <c r="Q21" s="2" t="n">
         <v>18800</v>
@@ -2226,14 +2064,6 @@
       <c r="S21" t="n">
         <v>0.02</v>
       </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U21" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2300,7 +2130,7 @@
         </is>
       </c>
       <c r="P22" t="n">
-        <v>1758.28</v>
+        <v>1723.8</v>
       </c>
       <c r="Q22" s="2" t="n">
         <v>18770</v>
@@ -2311,14 +2141,6 @@
       <c r="S22" t="n">
         <v>0.02</v>
       </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U22" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2385,7 +2207,7 @@
         </is>
       </c>
       <c r="P23" t="n">
-        <v>2892.31</v>
+        <v>2835.6</v>
       </c>
       <c r="Q23" s="2" t="n">
         <v>18452</v>
@@ -2396,14 +2218,6 @@
       <c r="S23" t="n">
         <v>0.02</v>
       </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U23" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2470,7 +2284,7 @@
         </is>
       </c>
       <c r="P24" t="n">
-        <v>1832.14</v>
+        <v>1796.22</v>
       </c>
       <c r="Q24" s="2" t="n">
         <v>22753</v>
@@ -2481,14 +2295,6 @@
       <c r="S24" t="n">
         <v>0.02</v>
       </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U24" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2555,7 +2361,7 @@
         </is>
       </c>
       <c r="P25" t="n">
-        <v>2100.57</v>
+        <v>2059.38</v>
       </c>
       <c r="Q25" s="2" t="n">
         <v>37446</v>
@@ -2566,14 +2372,6 @@
       <c r="S25" t="n">
         <v>0.02</v>
       </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U25" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2640,7 +2438,7 @@
         </is>
       </c>
       <c r="P26" t="n">
-        <v>2461.59</v>
+        <v>2413.32</v>
       </c>
       <c r="Q26" s="2" t="n">
         <v>20920</v>
@@ -2651,14 +2449,6 @@
       <c r="S26" t="n">
         <v>0.02</v>
       </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U26" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2725,7 +2515,7 @@
         </is>
       </c>
       <c r="P27" t="n">
-        <v>2273.27</v>
+        <v>2228.7</v>
       </c>
       <c r="Q27" s="2" t="n">
         <v>36364</v>
@@ -2736,14 +2526,6 @@
       <c r="S27" t="n">
         <v>0.02</v>
       </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U27" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2810,7 +2592,7 @@
         </is>
       </c>
       <c r="P28" t="n">
-        <v>2005.89</v>
+        <v>1966.56</v>
       </c>
       <c r="Q28" s="2" t="n">
         <v>23362</v>
@@ -2821,14 +2603,6 @@
       <c r="S28" t="n">
         <v>0.02</v>
       </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U28" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2895,7 +2669,7 @@
         </is>
       </c>
       <c r="P29" t="n">
-        <v>1832.14</v>
+        <v>1796.22</v>
       </c>
       <c r="Q29" s="2" t="n">
         <v>27820</v>
@@ -2906,14 +2680,6 @@
       <c r="S29" t="n">
         <v>0.02</v>
       </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U29" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2980,7 +2746,7 @@
         </is>
       </c>
       <c r="P30" t="n">
-        <v>2769.54</v>
+        <v>2715.24</v>
       </c>
       <c r="Q30" s="2" t="n">
         <v>25914</v>
@@ -2991,14 +2757,6 @@
       <c r="S30" t="n">
         <v>0.02</v>
       </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U30" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3065,7 +2823,7 @@
         </is>
       </c>
       <c r="P31" t="n">
-        <v>2386.68</v>
+        <v>2339.88</v>
       </c>
       <c r="Q31" s="2" t="n">
         <v>29103</v>
@@ -3076,14 +2834,6 @@
       <c r="S31" t="n">
         <v>0.02</v>
       </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U31" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3150,7 +2900,7 @@
         </is>
       </c>
       <c r="P32" t="n">
-        <v>2486.56</v>
+        <v>2437.8</v>
       </c>
       <c r="Q32" s="2" t="n">
         <v>31055</v>
@@ -3161,14 +2911,6 @@
       <c r="S32" t="n">
         <v>0.02</v>
       </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U32" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3235,7 +2977,7 @@
         </is>
       </c>
       <c r="P33" t="n">
-        <v>2712.32</v>
+        <v>2659.14</v>
       </c>
       <c r="Q33" s="2" t="n">
         <v>19160</v>
@@ -3246,14 +2988,6 @@
       <c r="S33" t="n">
         <v>0.02</v>
       </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U33" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3320,7 +3054,7 @@
         </is>
       </c>
       <c r="P34" t="n">
-        <v>1906.01</v>
+        <v>1868.64</v>
       </c>
       <c r="Q34" s="2" t="n">
         <v>30975</v>
@@ -3331,14 +3065,6 @@
       <c r="S34" t="n">
         <v>0.02</v>
       </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U34" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3405,7 +3131,7 @@
         </is>
       </c>
       <c r="P35" t="n">
-        <v>1767.64</v>
+        <v>1732.98</v>
       </c>
       <c r="Q35" s="2" t="n">
         <v>30825</v>
@@ -3416,14 +3142,6 @@
       <c r="S35" t="n">
         <v>0.02</v>
       </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U35" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3486,7 +3204,7 @@
         </is>
       </c>
       <c r="P36" t="n">
-        <v>2088.08</v>
+        <v>2047.14</v>
       </c>
       <c r="Q36" s="2" t="n">
         <v>34934</v>
@@ -3497,14 +3215,6 @@
       <c r="S36" t="n">
         <v>0.02</v>
       </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U36" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3567,7 +3277,7 @@
         </is>
       </c>
       <c r="P37" t="n">
-        <v>2913.12</v>
+        <v>2856</v>
       </c>
       <c r="Q37" s="2" t="n">
         <v>22234</v>
@@ -3578,14 +3288,6 @@
       <c r="S37" t="n">
         <v>0.02</v>
       </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U37" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3652,7 +3354,7 @@
         </is>
       </c>
       <c r="P38" t="n">
-        <v>2067.27</v>
+        <v>2026.74</v>
       </c>
       <c r="Q38" s="2" t="n">
         <v>33091</v>
@@ -3663,14 +3365,6 @@
       <c r="S38" t="n">
         <v>0.02</v>
       </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U38" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3737,7 +3431,7 @@
         </is>
       </c>
       <c r="P39" t="n">
-        <v>2823.65</v>
+        <v>2768.28</v>
       </c>
       <c r="Q39" s="2" t="n">
         <v>36096</v>
@@ -3748,14 +3442,6 @@
       <c r="S39" t="n">
         <v>0.02</v>
       </c>
-      <c r="T39" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U39" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3822,7 +3508,7 @@
         </is>
       </c>
       <c r="P40" t="n">
-        <v>2734.17</v>
+        <v>2680.56</v>
       </c>
       <c r="Q40" s="2" t="n">
         <v>34046</v>
@@ -3833,14 +3519,6 @@
       <c r="S40" t="n">
         <v>0.02</v>
       </c>
-      <c r="T40" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U40" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3907,7 +3585,7 @@
         </is>
       </c>
       <c r="P41" t="n">
-        <v>2673.83</v>
+        <v>2621.4</v>
       </c>
       <c r="Q41" s="2" t="n">
         <v>22242</v>
@@ -3918,14 +3596,6 @@
       <c r="S41" t="n">
         <v>0.02</v>
       </c>
-      <c r="T41" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U41" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3992,7 +3662,7 @@
         </is>
       </c>
       <c r="P42" t="n">
-        <v>2268.07</v>
+        <v>2223.6</v>
       </c>
       <c r="Q42" s="2" t="n">
         <v>21770</v>
@@ -4003,14 +3673,6 @@
       <c r="S42" t="n">
         <v>0.02</v>
       </c>
-      <c r="T42" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U42" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4077,7 +3739,7 @@
         </is>
       </c>
       <c r="P43" t="n">
-        <v>2900.64</v>
+        <v>2843.76</v>
       </c>
       <c r="Q43" s="2" t="n">
         <v>35467</v>
@@ -4088,14 +3750,6 @@
       <c r="S43" t="n">
         <v>0.02</v>
       </c>
-      <c r="T43" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U43" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4162,7 +3816,7 @@
         </is>
       </c>
       <c r="P44" t="n">
-        <v>1937.22</v>
+        <v>1899.24</v>
       </c>
       <c r="Q44" s="2" t="n">
         <v>35821</v>
@@ -4173,14 +3827,6 @@
       <c r="S44" t="n">
         <v>0.02</v>
       </c>
-      <c r="T44" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U44" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4247,7 +3893,7 @@
         </is>
       </c>
       <c r="P45" t="n">
-        <v>2721.69</v>
+        <v>2668.32</v>
       </c>
       <c r="Q45" s="2" t="n">
         <v>32043</v>
@@ -4258,14 +3904,6 @@
       <c r="S45" t="n">
         <v>0.02</v>
       </c>
-      <c r="T45" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U45" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4332,7 +3970,7 @@
         </is>
       </c>
       <c r="P46" t="n">
-        <v>2385.64</v>
+        <v>2338.86</v>
       </c>
       <c r="Q46" s="2" t="n">
         <v>23828</v>
@@ -4343,14 +3981,6 @@
       <c r="S46" t="n">
         <v>0.02</v>
       </c>
-      <c r="T46" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U46" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4417,7 +4047,7 @@
         </is>
       </c>
       <c r="P47" t="n">
-        <v>1918.5</v>
+        <v>1880.88</v>
       </c>
       <c r="Q47" s="2" t="n">
         <v>30936</v>
@@ -4428,14 +4058,6 @@
       <c r="S47" t="n">
         <v>0.02</v>
       </c>
-      <c r="T47" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U47" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4502,7 +4124,7 @@
         </is>
       </c>
       <c r="P48" t="n">
-        <v>1999.65</v>
+        <v>1960.44</v>
       </c>
       <c r="Q48" s="2" t="n">
         <v>19969</v>
@@ -4513,14 +4135,6 @@
       <c r="S48" t="n">
         <v>0.02</v>
       </c>
-      <c r="T48" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U48" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4587,7 +4201,7 @@
         </is>
       </c>
       <c r="P49" t="n">
-        <v>2337.78</v>
+        <v>2291.94</v>
       </c>
       <c r="Q49" s="2" t="n">
         <v>24097</v>
@@ -4598,14 +4212,6 @@
       <c r="S49" t="n">
         <v>0.02</v>
       </c>
-      <c r="T49" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U49" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4672,7 +4278,7 @@
         </is>
       </c>
       <c r="P50" t="n">
-        <v>2116.17</v>
+        <v>2074.68</v>
       </c>
       <c r="Q50" s="2" t="n">
         <v>19346</v>
@@ -4683,14 +4289,6 @@
       <c r="S50" t="n">
         <v>0.02</v>
       </c>
-      <c r="T50" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U50" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4757,7 +4355,7 @@
         </is>
       </c>
       <c r="P51" t="n">
-        <v>2143.22</v>
+        <v>2101.2</v>
       </c>
       <c r="Q51" s="2" t="n">
         <v>22254</v>
@@ -4768,14 +4366,6 @@
       <c r="S51" t="n">
         <v>0.02</v>
       </c>
-      <c r="T51" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U51" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4842,7 +4432,7 @@
         </is>
       </c>
       <c r="P52" t="n">
-        <v>2026.7</v>
+        <v>1986.96</v>
       </c>
       <c r="Q52" s="2" t="n">
         <v>28829</v>
@@ -4853,14 +4443,6 @@
       <c r="S52" t="n">
         <v>0.02</v>
       </c>
-      <c r="T52" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U52" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4927,23 +4509,15 @@
         </is>
       </c>
       <c r="P53" t="n">
-        <v>2585.39</v>
+        <v>2534.7</v>
       </c>
       <c r="Q53" s="2" t="n">
         <v>27813</v>
       </c>
       <c r="R53" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S53" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="T53" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U53" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -5012,7 +4586,7 @@
         </is>
       </c>
       <c r="P54" t="n">
-        <v>2971.38</v>
+        <v>2913.12</v>
       </c>
       <c r="Q54" s="2" t="n">
         <v>34824</v>
@@ -5023,14 +4597,6 @@
       <c r="S54" t="n">
         <v>0.02</v>
       </c>
-      <c r="T54" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U54" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5097,7 +4663,7 @@
         </is>
       </c>
       <c r="P55" t="n">
-        <v>2440.78</v>
+        <v>2392.92</v>
       </c>
       <c r="Q55" s="2" t="n">
         <v>25915</v>
@@ -5108,14 +4674,6 @@
       <c r="S55" t="n">
         <v>0.02</v>
       </c>
-      <c r="T55" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U55" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5182,7 +4740,7 @@
         </is>
       </c>
       <c r="P56" t="n">
-        <v>2455.34</v>
+        <v>2407.2</v>
       </c>
       <c r="Q56" s="2" t="n">
         <v>22324</v>
@@ -5193,14 +4751,6 @@
       <c r="S56" t="n">
         <v>0.02</v>
       </c>
-      <c r="T56" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U56" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5267,7 +4817,7 @@
         </is>
       </c>
       <c r="P57" t="n">
-        <v>2097.45</v>
+        <v>2056.32</v>
       </c>
       <c r="Q57" s="2" t="n">
         <v>19749</v>
@@ -5278,14 +4828,6 @@
       <c r="S57" t="n">
         <v>0.02</v>
       </c>
-      <c r="T57" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U57" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5352,7 +4894,7 @@
         </is>
       </c>
       <c r="P58" t="n">
-        <v>2735.21</v>
+        <v>2681.58</v>
       </c>
       <c r="Q58" s="2" t="n">
         <v>32102</v>
@@ -5363,14 +4905,6 @@
       <c r="S58" t="n">
         <v>0.02</v>
       </c>
-      <c r="T58" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U58" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5437,7 +4971,7 @@
         </is>
       </c>
       <c r="P59" t="n">
-        <v>2466.79</v>
+        <v>2418.42</v>
       </c>
       <c r="Q59" s="2" t="n">
         <v>20100</v>
@@ -5448,14 +4982,6 @@
       <c r="S59" t="n">
         <v>0.02</v>
       </c>
-      <c r="T59" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U59" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5518,7 +5044,7 @@
         </is>
       </c>
       <c r="P60" t="n">
-        <v>2146.35</v>
+        <v>2104.26</v>
       </c>
       <c r="Q60" s="2" t="n">
         <v>23569</v>
@@ -5529,14 +5055,6 @@
       <c r="S60" t="n">
         <v>0.02</v>
       </c>
-      <c r="T60" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U60" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5603,7 +5121,7 @@
         </is>
       </c>
       <c r="P61" t="n">
-        <v>2175.48</v>
+        <v>2132.82</v>
       </c>
       <c r="Q61" s="2" t="n">
         <v>37172</v>
@@ -5614,14 +5132,6 @@
       <c r="S61" t="n">
         <v>0.02</v>
       </c>
-      <c r="T61" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U61" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5688,7 +5198,7 @@
         </is>
       </c>
       <c r="P62" t="n">
-        <v>2263.91</v>
+        <v>2219.52</v>
       </c>
       <c r="Q62" s="2" t="n">
         <v>20381</v>
@@ -5699,14 +5209,6 @@
       <c r="S62" t="n">
         <v>0.02</v>
       </c>
-      <c r="T62" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U62" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5773,7 +5275,7 @@
         </is>
       </c>
       <c r="P63" t="n">
-        <v>2831.97</v>
+        <v>2776.44</v>
       </c>
       <c r="Q63" s="2" t="n">
         <v>32483</v>
@@ -5784,14 +5286,6 @@
       <c r="S63" t="n">
         <v>0.02</v>
       </c>
-      <c r="T63" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U63" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5858,7 +5352,7 @@
         </is>
       </c>
       <c r="P64" t="n">
-        <v>2244.14</v>
+        <v>2200.14</v>
       </c>
       <c r="Q64" s="2" t="n">
         <v>23322</v>
@@ -5869,14 +5363,6 @@
       <c r="S64" t="n">
         <v>0.02</v>
       </c>
-      <c r="T64" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U64" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5943,7 +5429,7 @@
         </is>
       </c>
       <c r="P65" t="n">
-        <v>2846.53</v>
+        <v>2790.72</v>
       </c>
       <c r="Q65" s="2" t="n">
         <v>31224</v>
@@ -5954,14 +5440,6 @@
       <c r="S65" t="n">
         <v>0.02</v>
       </c>
-      <c r="T65" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U65" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -6028,7 +5506,7 @@
         </is>
       </c>
       <c r="P66" t="n">
-        <v>2645.74</v>
+        <v>2593.86</v>
       </c>
       <c r="Q66" s="2" t="n">
         <v>31751</v>
@@ -6039,14 +5517,6 @@
       <c r="S66" t="n">
         <v>0.02</v>
       </c>
-      <c r="T66" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U66" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6113,7 +5583,7 @@
         </is>
       </c>
       <c r="P67" t="n">
-        <v>2074.56</v>
+        <v>2033.88</v>
       </c>
       <c r="Q67" s="2" t="n">
         <v>23933</v>
@@ -6124,14 +5594,6 @@
       <c r="S67" t="n">
         <v>0.02</v>
       </c>
-      <c r="T67" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U67" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6198,7 +5660,7 @@
         </is>
       </c>
       <c r="P68" t="n">
-        <v>2306.57</v>
+        <v>2261.34</v>
       </c>
       <c r="Q68" s="2" t="n">
         <v>28092</v>
@@ -6209,14 +5671,6 @@
       <c r="S68" t="n">
         <v>0.02</v>
       </c>
-      <c r="T68" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U68" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6283,7 +5737,7 @@
         </is>
       </c>
       <c r="P69" t="n">
-        <v>2618.69</v>
+        <v>2567.34</v>
       </c>
       <c r="Q69" s="2" t="n">
         <v>33550</v>
@@ -6294,14 +5748,6 @@
       <c r="S69" t="n">
         <v>0.02</v>
       </c>
-      <c r="T69" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U69" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6368,7 +5814,7 @@
         </is>
       </c>
       <c r="P70" t="n">
-        <v>2404.36</v>
+        <v>2357.22</v>
       </c>
       <c r="Q70" s="2" t="n">
         <v>23575</v>
@@ -6379,14 +5825,6 @@
       <c r="S70" t="n">
         <v>0.02</v>
       </c>
-      <c r="T70" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U70" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6453,7 +5891,7 @@
         </is>
       </c>
       <c r="P71" t="n">
-        <v>2314.89</v>
+        <v>2269.5</v>
       </c>
       <c r="Q71" s="2" t="n">
         <v>26641</v>
@@ -6464,14 +5902,6 @@
       <c r="S71" t="n">
         <v>0.02</v>
       </c>
-      <c r="T71" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U71" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6538,7 +5968,7 @@
         </is>
       </c>
       <c r="P72" t="n">
-        <v>2375.23</v>
+        <v>2328.66</v>
       </c>
       <c r="Q72" s="2" t="n">
         <v>28566</v>
@@ -6549,14 +5979,6 @@
       <c r="S72" t="n">
         <v>0.02</v>
       </c>
-      <c r="T72" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U72" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6623,7 +6045,7 @@
         </is>
       </c>
       <c r="P73" t="n">
-        <v>2042.31</v>
+        <v>2002.26</v>
       </c>
       <c r="Q73" s="2" t="n">
         <v>37088</v>
@@ -6634,14 +6056,6 @@
       <c r="S73" t="n">
         <v>0.02</v>
       </c>
-      <c r="T73" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U73" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6708,7 +6122,7 @@
         </is>
       </c>
       <c r="P74" t="n">
-        <v>2611.4</v>
+        <v>2560.2</v>
       </c>
       <c r="Q74" s="2" t="n">
         <v>29647</v>
@@ -6719,14 +6133,6 @@
       <c r="S74" t="n">
         <v>0.02</v>
       </c>
-      <c r="T74" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U74" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6793,7 +6199,7 @@
         </is>
       </c>
       <c r="P75" t="n">
-        <v>2957.86</v>
+        <v>2899.86</v>
       </c>
       <c r="Q75" s="2" t="n">
         <v>35182</v>
@@ -6804,14 +6210,6 @@
       <c r="S75" t="n">
         <v>0.02</v>
       </c>
-      <c r="T75" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U75" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6878,7 +6276,7 @@
         </is>
       </c>
       <c r="P76" t="n">
-        <v>2409.57</v>
+        <v>2362.32</v>
       </c>
       <c r="Q76" s="2" t="n">
         <v>25915</v>
@@ -6889,14 +6287,6 @@
       <c r="S76" t="n">
         <v>0.02</v>
       </c>
-      <c r="T76" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U76" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6963,7 +6353,7 @@
         </is>
       </c>
       <c r="P77" t="n">
-        <v>1814.46</v>
+        <v>1778.88</v>
       </c>
       <c r="Q77" s="2" t="n">
         <v>28705</v>
@@ -6974,14 +6364,6 @@
       <c r="S77" t="n">
         <v>0.02</v>
       </c>
-      <c r="T77" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U77" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -7048,7 +6430,7 @@
         </is>
       </c>
       <c r="P78" t="n">
-        <v>2710.24</v>
+        <v>2657.1</v>
       </c>
       <c r="Q78" s="2" t="n">
         <v>23663</v>
@@ -7059,14 +6441,6 @@
       <c r="S78" t="n">
         <v>0.02</v>
       </c>
-      <c r="T78" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U78" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7129,7 +6503,7 @@
         </is>
       </c>
       <c r="P79" t="n">
-        <v>2520.89</v>
+        <v>2471.46</v>
       </c>
       <c r="Q79" s="2" t="n">
         <v>25403</v>
@@ -7140,14 +6514,6 @@
       <c r="S79" t="n">
         <v>0.02</v>
       </c>
-      <c r="T79" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U79" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -7214,7 +6580,7 @@
         </is>
       </c>
       <c r="P80" t="n">
-        <v>2628.05</v>
+        <v>2576.52</v>
       </c>
       <c r="Q80" s="2" t="n">
         <v>37076</v>
@@ -7225,14 +6591,6 @@
       <c r="S80" t="n">
         <v>0.02</v>
       </c>
-      <c r="T80" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U80" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7299,7 +6657,7 @@
         </is>
       </c>
       <c r="P81" t="n">
-        <v>2489.68</v>
+        <v>2440.86</v>
       </c>
       <c r="Q81" s="2" t="n">
         <v>36515</v>
@@ -7310,14 +6668,6 @@
       <c r="S81" t="n">
         <v>0.02</v>
       </c>
-      <c r="T81" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U81" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -7384,7 +6734,7 @@
         </is>
       </c>
       <c r="P82" t="n">
-        <v>1872.72</v>
+        <v>1836</v>
       </c>
       <c r="Q82" s="2" t="n">
         <v>31489</v>
@@ -7395,14 +6745,6 @@
       <c r="S82" t="n">
         <v>0.02</v>
       </c>
-      <c r="T82" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U82" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -7469,7 +6811,7 @@
         </is>
       </c>
       <c r="P83" t="n">
-        <v>2152.59</v>
+        <v>2110.38</v>
       </c>
       <c r="Q83" s="2" t="n">
         <v>24789</v>
@@ -7480,14 +6822,6 @@
       <c r="S83" t="n">
         <v>0.02</v>
       </c>
-      <c r="T83" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U83" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -7554,7 +6888,7 @@
         </is>
       </c>
       <c r="P84" t="n">
-        <v>2143.22</v>
+        <v>2101.2</v>
       </c>
       <c r="Q84" s="2" t="n">
         <v>20343</v>
@@ -7565,14 +6899,6 @@
       <c r="S84" t="n">
         <v>0.02</v>
       </c>
-      <c r="T84" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U84" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7639,7 +6965,7 @@
         </is>
       </c>
       <c r="P85" t="n">
-        <v>1918.5</v>
+        <v>1880.88</v>
       </c>
       <c r="Q85" s="2" t="n">
         <v>22800</v>
@@ -7650,14 +6976,6 @@
       <c r="S85" t="n">
         <v>0.02</v>
       </c>
-      <c r="T85" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U85" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7724,7 +7042,7 @@
         </is>
       </c>
       <c r="P86" t="n">
-        <v>1858.15</v>
+        <v>1821.72</v>
       </c>
       <c r="Q86" s="2" t="n">
         <v>18995</v>
@@ -7735,14 +7053,6 @@
       <c r="S86" t="n">
         <v>0.02</v>
       </c>
-      <c r="T86" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U86" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7809,23 +7119,15 @@
         </is>
       </c>
       <c r="P87" t="n">
-        <v>1801.97</v>
+        <v>1766.64</v>
       </c>
       <c r="Q87" s="2" t="n">
         <v>19781</v>
       </c>
       <c r="R87" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="S87" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="T87" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U87" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -7890,7 +7192,7 @@
         </is>
       </c>
       <c r="P88" t="n">
-        <v>1909.13</v>
+        <v>1871.7</v>
       </c>
       <c r="Q88" s="2" t="n">
         <v>34444</v>
@@ -7901,14 +7203,6 @@
       <c r="S88" t="n">
         <v>0.02</v>
       </c>
-      <c r="T88" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U88" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7975,7 +7269,7 @@
         </is>
       </c>
       <c r="P89" t="n">
-        <v>2251.43</v>
+        <v>2207.28</v>
       </c>
       <c r="Q89" s="2" t="n">
         <v>36671</v>
@@ -7986,14 +7280,6 @@
       <c r="S89" t="n">
         <v>0.02</v>
       </c>
-      <c r="T89" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U89" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -8060,7 +7346,7 @@
         </is>
       </c>
       <c r="P90" t="n">
-        <v>2641.58</v>
+        <v>2589.78</v>
       </c>
       <c r="Q90" s="2" t="n">
         <v>21243</v>
@@ -8071,14 +7357,6 @@
       <c r="S90" t="n">
         <v>0.02</v>
       </c>
-      <c r="T90" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U90" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -8145,7 +7423,7 @@
         </is>
       </c>
       <c r="P91" t="n">
-        <v>1980.92</v>
+        <v>1942.08</v>
       </c>
       <c r="Q91" s="2" t="n">
         <v>19308</v>
@@ -8156,14 +7434,6 @@
       <c r="S91" t="n">
         <v>0.02</v>
       </c>
-      <c r="T91" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U91" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -8230,7 +7500,7 @@
         </is>
       </c>
       <c r="P92" t="n">
-        <v>2840.29</v>
+        <v>2784.6</v>
       </c>
       <c r="Q92" s="2" t="n">
         <v>31941</v>
@@ -8241,14 +7511,6 @@
       <c r="S92" t="n">
         <v>0.02</v>
       </c>
-      <c r="T92" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U92" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8315,7 +7577,7 @@
         </is>
       </c>
       <c r="P93" t="n">
-        <v>2930.81</v>
+        <v>2873.34</v>
       </c>
       <c r="Q93" s="2" t="n">
         <v>27906</v>
@@ -8326,14 +7588,6 @@
       <c r="S93" t="n">
         <v>0.02</v>
       </c>
-      <c r="T93" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U93" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -8400,7 +7654,7 @@
         </is>
       </c>
       <c r="P94" t="n">
-        <v>2041.26</v>
+        <v>2001.24</v>
       </c>
       <c r="Q94" s="2" t="n">
         <v>20339</v>
@@ -8411,14 +7665,6 @@
       <c r="S94" t="n">
         <v>0.02</v>
       </c>
-      <c r="T94" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U94" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -8485,7 +7731,7 @@
         </is>
       </c>
       <c r="P95" t="n">
-        <v>2876.71</v>
+        <v>2820.3</v>
       </c>
       <c r="Q95" s="2" t="n">
         <v>19652</v>
@@ -8496,14 +7742,6 @@
       <c r="S95" t="n">
         <v>0.02</v>
       </c>
-      <c r="T95" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U95" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -8566,7 +7804,7 @@
         </is>
       </c>
       <c r="P96" t="n">
-        <v>2039.18</v>
+        <v>1999.2</v>
       </c>
       <c r="Q96" s="2" t="n">
         <v>23697</v>
@@ -8577,14 +7815,6 @@
       <c r="S96" t="n">
         <v>0.02</v>
       </c>
-      <c r="T96" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U96" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -8651,7 +7881,7 @@
         </is>
       </c>
       <c r="P97" t="n">
-        <v>2028.78</v>
+        <v>1989</v>
       </c>
       <c r="Q97" s="2" t="n">
         <v>23569</v>
@@ -8662,14 +7892,6 @@
       <c r="S97" t="n">
         <v>0.02</v>
       </c>
-      <c r="T97" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U97" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8736,7 +7958,7 @@
         </is>
       </c>
       <c r="P98" t="n">
-        <v>1977.8</v>
+        <v>1939.02</v>
       </c>
       <c r="Q98" s="2" t="n">
         <v>27038</v>
@@ -8747,14 +7969,6 @@
       <c r="S98" t="n">
         <v>0.02</v>
       </c>
-      <c r="T98" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U98" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8821,7 +8035,7 @@
         </is>
       </c>
       <c r="P99" t="n">
-        <v>2350.26</v>
+        <v>2304.18</v>
       </c>
       <c r="Q99" s="2" t="n">
         <v>31760</v>
@@ -8832,14 +8046,6 @@
       <c r="S99" t="n">
         <v>0.02</v>
       </c>
-      <c r="T99" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U99" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8906,7 +8112,7 @@
         </is>
       </c>
       <c r="P100" t="n">
-        <v>1676.08</v>
+        <v>1643.22</v>
       </c>
       <c r="Q100" s="2" t="n">
         <v>27092</v>
@@ -8917,14 +8123,6 @@
       <c r="S100" t="n">
         <v>0.02</v>
       </c>
-      <c r="T100" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U100" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8991,7 +8189,7 @@
         </is>
       </c>
       <c r="P101" t="n">
-        <v>2455.34</v>
+        <v>2407.2</v>
       </c>
       <c r="Q101" s="2" t="n">
         <v>38526</v>
@@ -9002,14 +8200,6 @@
       <c r="S101" t="n">
         <v>0.02</v>
       </c>
-      <c r="T101" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U101" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -9076,7 +8266,7 @@
         </is>
       </c>
       <c r="P102" t="n">
-        <v>2651.98</v>
+        <v>2599.98</v>
       </c>
       <c r="Q102" s="2" t="n">
         <v>33859</v>
@@ -9087,14 +8277,6 @@
       <c r="S102" t="n">
         <v>0.02</v>
       </c>
-      <c r="T102" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U102" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -9161,7 +8343,7 @@
         </is>
       </c>
       <c r="P103" t="n">
-        <v>2918.32</v>
+        <v>2861.1</v>
       </c>
       <c r="Q103" s="2" t="n">
         <v>32143</v>
@@ -9172,14 +8354,6 @@
       <c r="S103" t="n">
         <v>0.02</v>
       </c>
-      <c r="T103" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U103" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -9246,7 +8420,7 @@
         </is>
       </c>
       <c r="P104" t="n">
-        <v>1593.89</v>
+        <v>1562.64</v>
       </c>
       <c r="Q104" s="2" t="n">
         <v>21522</v>
@@ -9257,14 +8431,6 @@
       <c r="S104" t="n">
         <v>0.02</v>
       </c>
-      <c r="T104" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U104" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -9331,7 +8497,7 @@
         </is>
       </c>
       <c r="P105" t="n">
-        <v>2419.97</v>
+        <v>2372.52</v>
       </c>
       <c r="Q105" s="2" t="n">
         <v>22873</v>
@@ -9342,14 +8508,6 @@
       <c r="S105" t="n">
         <v>0.02</v>
       </c>
-      <c r="T105" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U105" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -9416,7 +8574,7 @@
         </is>
       </c>
       <c r="P106" t="n">
-        <v>2229.58</v>
+        <v>2185.86</v>
       </c>
       <c r="Q106" s="2" t="n">
         <v>24979</v>
@@ -9427,14 +8585,6 @@
       <c r="S106" t="n">
         <v>0.02</v>
       </c>
-      <c r="T106" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U106" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -9501,7 +8651,7 @@
         </is>
       </c>
       <c r="P107" t="n">
-        <v>2502.16</v>
+        <v>2453.1</v>
       </c>
       <c r="Q107" s="2" t="n">
         <v>21840</v>
@@ -9512,14 +8662,6 @@
       <c r="S107" t="n">
         <v>0.02</v>
       </c>
-      <c r="T107" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U107" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -9586,7 +8728,7 @@
         </is>
       </c>
       <c r="P108" t="n">
-        <v>2487.6</v>
+        <v>2438.82</v>
       </c>
       <c r="Q108" s="2" t="n">
         <v>24641</v>
@@ -9597,14 +8739,6 @@
       <c r="S108" t="n">
         <v>0.02</v>
       </c>
-      <c r="T108" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U108" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -9671,7 +8805,7 @@
         </is>
       </c>
       <c r="P109" t="n">
-        <v>1813.42</v>
+        <v>1777.86</v>
       </c>
       <c r="Q109" s="2" t="n">
         <v>34234</v>
@@ -9682,14 +8816,6 @@
       <c r="S109" t="n">
         <v>0.02</v>
       </c>
-      <c r="T109" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U109" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -9756,7 +8882,7 @@
         </is>
       </c>
       <c r="P110" t="n">
-        <v>2131.78</v>
+        <v>2089.98</v>
       </c>
       <c r="Q110" s="2" t="n">
         <v>23210</v>
@@ -9767,14 +8893,6 @@
       <c r="S110" t="n">
         <v>0.02</v>
       </c>
-      <c r="T110" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U110" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9841,23 +8959,15 @@
         </is>
       </c>
       <c r="P111" t="n">
-        <v>2615.57</v>
+        <v>2564.28</v>
       </c>
       <c r="Q111" s="2" t="n">
         <v>25624</v>
       </c>
       <c r="R111" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="S111" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="T111" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U111" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -9926,7 +9036,7 @@
         </is>
       </c>
       <c r="P112" t="n">
-        <v>2486.56</v>
+        <v>2437.8</v>
       </c>
       <c r="Q112" s="2" t="n">
         <v>36586</v>
@@ -9937,14 +9047,6 @@
       <c r="S112" t="n">
         <v>0.02</v>
       </c>
-      <c r="T112" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U112" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -10011,7 +9113,7 @@
         </is>
       </c>
       <c r="P113" t="n">
-        <v>2445.98</v>
+        <v>2398.02</v>
       </c>
       <c r="Q113" s="2" t="n">
         <v>26241</v>
@@ -10022,14 +9124,6 @@
       <c r="S113" t="n">
         <v>0.02</v>
       </c>
-      <c r="T113" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U113" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -10096,7 +9190,7 @@
         </is>
       </c>
       <c r="P114" t="n">
-        <v>2005.89</v>
+        <v>1966.56</v>
       </c>
       <c r="Q114" s="2" t="n">
         <v>28684</v>
@@ -10107,14 +9201,6 @@
       <c r="S114" t="n">
         <v>0.02</v>
       </c>
-      <c r="T114" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U114" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -10181,7 +9267,7 @@
         </is>
       </c>
       <c r="P115" t="n">
-        <v>2289.92</v>
+        <v>2245.02</v>
       </c>
       <c r="Q115" s="2" t="n">
         <v>25850</v>
@@ -10192,14 +9278,6 @@
       <c r="S115" t="n">
         <v>0.02</v>
       </c>
-      <c r="T115" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U115" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -10266,7 +9344,7 @@
         </is>
       </c>
       <c r="P116" t="n">
-        <v>2399.16</v>
+        <v>2352.12</v>
       </c>
       <c r="Q116" s="2" t="n">
         <v>26665</v>
@@ -10277,14 +9355,6 @@
       <c r="S116" t="n">
         <v>0.02</v>
       </c>
-      <c r="T116" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U116" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -10351,7 +9421,7 @@
         </is>
       </c>
       <c r="P117" t="n">
-        <v>3029.64</v>
+        <v>2970.24</v>
       </c>
       <c r="Q117" s="2" t="n">
         <v>30670</v>
@@ -10362,14 +9432,6 @@
       <c r="S117" t="n">
         <v>0.02</v>
       </c>
-      <c r="T117" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U117" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -10436,7 +9498,7 @@
         </is>
       </c>
       <c r="P118" t="n">
-        <v>2346.1</v>
+        <v>2300.1</v>
       </c>
       <c r="Q118" s="2" t="n">
         <v>24670</v>
@@ -10447,14 +9509,6 @@
       <c r="S118" t="n">
         <v>0.02</v>
       </c>
-      <c r="T118" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U118" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -10521,7 +9575,7 @@
         </is>
       </c>
       <c r="P119" t="n">
-        <v>1945.55</v>
+        <v>1907.4</v>
       </c>
       <c r="Q119" s="2" t="n">
         <v>18601</v>
@@ -10532,14 +9586,6 @@
       <c r="S119" t="n">
         <v>0.02</v>
       </c>
-      <c r="T119" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U119" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10606,7 +9652,7 @@
         </is>
       </c>
       <c r="P120" t="n">
-        <v>2545.86</v>
+        <v>2495.94</v>
       </c>
       <c r="Q120" s="2" t="n">
         <v>37962</v>
@@ -10617,14 +9663,6 @@
       <c r="S120" t="n">
         <v>0.02</v>
       </c>
-      <c r="T120" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U120" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10691,7 +9729,7 @@
         </is>
       </c>
       <c r="P121" t="n">
-        <v>1764.52</v>
+        <v>1729.92</v>
       </c>
       <c r="Q121" s="2" t="n">
         <v>26610</v>
@@ -10702,14 +9740,6 @@
       <c r="S121" t="n">
         <v>0.02</v>
       </c>
-      <c r="T121" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U121" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10776,7 +9806,7 @@
         </is>
       </c>
       <c r="P122" t="n">
-        <v>2192.12</v>
+        <v>2149.14</v>
       </c>
       <c r="Q122" s="2" t="n">
         <v>21832</v>
@@ -10787,14 +9817,6 @@
       <c r="S122" t="n">
         <v>0.02</v>
       </c>
-      <c r="T122" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U122" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10861,7 +9883,7 @@
         </is>
       </c>
       <c r="P123" t="n">
-        <v>2451.18</v>
+        <v>2403.12</v>
       </c>
       <c r="Q123" s="2" t="n">
         <v>29348</v>
@@ -10872,14 +9894,6 @@
       <c r="S123" t="n">
         <v>0.02</v>
       </c>
-      <c r="T123" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U123" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10946,7 +9960,7 @@
         </is>
       </c>
       <c r="P124" t="n">
-        <v>2259.75</v>
+        <v>2215.44</v>
       </c>
       <c r="Q124" s="2" t="n">
         <v>30661</v>
@@ -10957,14 +9971,6 @@
       <c r="S124" t="n">
         <v>0.02</v>
       </c>
-      <c r="T124" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U124" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -11031,7 +10037,7 @@
         </is>
       </c>
       <c r="P125" t="n">
-        <v>2006.93</v>
+        <v>1967.58</v>
       </c>
       <c r="Q125" s="2" t="n">
         <v>24269</v>
@@ -11042,14 +10048,6 @@
       <c r="S125" t="n">
         <v>0.02</v>
       </c>
-      <c r="T125" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U125" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -11116,7 +10114,7 @@
         </is>
       </c>
       <c r="P126" t="n">
-        <v>2510.49</v>
+        <v>2461.26</v>
       </c>
       <c r="Q126" s="2" t="n">
         <v>23038</v>
@@ -11127,14 +10125,6 @@
       <c r="S126" t="n">
         <v>0.02</v>
       </c>
-      <c r="T126" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U126" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -11201,7 +10191,7 @@
         </is>
       </c>
       <c r="P127" t="n">
-        <v>1935.14</v>
+        <v>1897.2</v>
       </c>
       <c r="Q127" s="2" t="n">
         <v>30841</v>
@@ -11212,14 +10202,6 @@
       <c r="S127" t="n">
         <v>0.02</v>
       </c>
-      <c r="T127" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U127" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -11286,7 +10268,7 @@
         </is>
       </c>
       <c r="P128" t="n">
-        <v>2387.72</v>
+        <v>2340.9</v>
       </c>
       <c r="Q128" s="2" t="n">
         <v>28759</v>
@@ -11297,14 +10279,6 @@
       <c r="S128" t="n">
         <v>0.02</v>
       </c>
-      <c r="T128" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U128" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -11371,7 +10345,7 @@
         </is>
       </c>
       <c r="P129" t="n">
-        <v>1897.69</v>
+        <v>1860.48</v>
       </c>
       <c r="Q129" s="2" t="n">
         <v>34611</v>
@@ -11382,14 +10356,6 @@
       <c r="S129" t="n">
         <v>0.02</v>
       </c>
-      <c r="T129" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U129" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -11456,7 +10422,7 @@
         </is>
       </c>
       <c r="P130" t="n">
-        <v>2339.86</v>
+        <v>2293.98</v>
       </c>
       <c r="Q130" s="2" t="n">
         <v>28752</v>
@@ -11467,14 +10433,6 @@
       <c r="S130" t="n">
         <v>0.02</v>
       </c>
-      <c r="T130" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U130" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -11541,7 +10499,7 @@
         </is>
       </c>
       <c r="P131" t="n">
-        <v>1620.94</v>
+        <v>1589.16</v>
       </c>
       <c r="Q131" s="2" t="n">
         <v>29279</v>
@@ -11552,14 +10510,6 @@
       <c r="S131" t="n">
         <v>0.02</v>
       </c>
-      <c r="T131" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U131" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -11626,7 +10576,7 @@
         </is>
       </c>
       <c r="P132" t="n">
-        <v>1970.52</v>
+        <v>1931.88</v>
       </c>
       <c r="Q132" s="2" t="n">
         <v>18696</v>
@@ -11637,14 +10587,6 @@
       <c r="S132" t="n">
         <v>0.02</v>
       </c>
-      <c r="T132" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U132" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -11711,7 +10653,7 @@
         </is>
       </c>
       <c r="P133" t="n">
-        <v>2557.3</v>
+        <v>2507.16</v>
       </c>
       <c r="Q133" s="2" t="n">
         <v>33586</v>
@@ -11722,14 +10664,6 @@
       <c r="S133" t="n">
         <v>0.02</v>
       </c>
-      <c r="T133" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U133" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -11796,7 +10730,7 @@
         </is>
       </c>
       <c r="P134" t="n">
-        <v>1593.89</v>
+        <v>1562.64</v>
       </c>
       <c r="Q134" s="2" t="n">
         <v>20587</v>
@@ -11807,14 +10741,6 @@
       <c r="S134" t="n">
         <v>0.02</v>
       </c>
-      <c r="T134" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U134" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -11881,7 +10807,7 @@
         </is>
       </c>
       <c r="P135" t="n">
-        <v>2559.38</v>
+        <v>2509.2</v>
       </c>
       <c r="Q135" s="2" t="n">
         <v>23762</v>
@@ -11892,14 +10818,6 @@
       <c r="S135" t="n">
         <v>0.02</v>
       </c>
-      <c r="T135" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U135" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -11966,7 +10884,7 @@
         </is>
       </c>
       <c r="P136" t="n">
-        <v>2372.11</v>
+        <v>2325.6</v>
       </c>
       <c r="Q136" s="2" t="n">
         <v>19788</v>
@@ -11977,14 +10895,6 @@
       <c r="S136" t="n">
         <v>0.02</v>
       </c>
-      <c r="T136" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U136" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -12051,7 +10961,7 @@
         </is>
       </c>
       <c r="P137" t="n">
-        <v>2256.63</v>
+        <v>2212.38</v>
       </c>
       <c r="Q137" s="2" t="n">
         <v>33505</v>
@@ -12062,14 +10972,6 @@
       <c r="S137" t="n">
         <v>0.02</v>
       </c>
-      <c r="T137" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U137" t="n">
-        <v>0.02</v>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -12136,7 +11038,7 @@
         </is>
       </c>
       <c r="P138" t="n">
-        <v>2277.44</v>
+        <v>2232.78</v>
       </c>
       <c r="Q138" s="2" t="n">
         <v>30453</v>
@@ -12145,14 +11047,6 @@
         <v>42</v>
       </c>
       <c r="S138" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="T138" t="inlineStr">
-        <is>
-          <t>2%</t>
-        </is>
-      </c>
-      <c r="U138" t="n">
         <v>0.02</v>
       </c>
     </row>

</xml_diff>